<commit_message>
Add ML classifier comparison and benchmark pipeline
</commit_message>
<xml_diff>
--- a/classifier/data/processed/labeled.xlsx
+++ b/classifier/data/processed/labeled.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -2242,6 +2242,1806 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>What is the tallest mountain in the world?</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>고양이는 영어로 뭐야?</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>번역</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>How many days are in a leap year?</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>파이썬에서 주석은 어떻게 써?</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>단순 사용법</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>What is the square root of 144?</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>단순 계산</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>냉장고 발명한 사람이 누구야?</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>What does 'RAM' stand for?</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>약어 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>사람의 정상 체온은 몇 도야?</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>What programming language is used for iOS development?</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>'사랑해'를 프랑스어로 번역해줘.</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>번역</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>What is the capital of Japan?</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>배열의 인덱스는 몇 번부터 시작해?</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>What is 7 times 8?</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>단순 계산</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>지구의 자전 주기는 얼마야?</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>What does 'CSS' stand for?</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>약어 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>한국의 화폐 단위가 뭐야?</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Who created the Python programming language?</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>리스트에서 마지막 요소를 꺼내는 파이썬 메서드는?</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>단순 사용법</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>What is the largest ocean on Earth?</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>오늘 날씨 어때? 라는 말을 영어로 해줘.</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>번역</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>What is a function in programming?</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>HTTP와 HTTPS의 차이가 뭐야?</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>단순 비교</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>What year did World War II end?</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>파이썬 딕셔너리에서 키를 꺼내는 방법은?</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>단순 사용법</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>What is the SI unit of electric current?</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>재귀함수가 뭐야?</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>What is the speed of light in km/s?</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>클라우드 컴퓨팅이 뭔지 한 줄로 설명해줘.</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>단순 요약</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Who is the author of Harry Potter?</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SQL에서 데이터를 조회할 때 쓰는 명령어는?</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>What is the difference between a compiler and an interpreter?</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>단순 비교</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>빅데이터의 3V가 뭐야?</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>What does 'URL' stand for?</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>약어 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>파이썬에서 for문 기본 문법이 어떻게 돼?</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>단순 사용법</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>What is the atomic number of carbon?</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>단순 사실</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>REST API가 뭐야?</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>What is Newton's first law of motion?</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>JSON이 뭐야?</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>What is the binary representation of the number 10?</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>0</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>단순 계산</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>깃(Git)에서 커밋이 뭐야?</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>What is a database index?</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>OOP에서 상속이 뭐야?</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>What does 'IP' stand for in IP address?</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>약어 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>파이썬에서 None이 뭐야?</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>0</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>What is a boolean data type?</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>0</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>도커(Docker)가 뭔지 한 줄로 설명해줘.</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>0</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>단순 요약</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>What is the difference between stack and queue?</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>단순 비교</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>API 키가 뭐야?</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>What is a hash function?</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>단순 정의</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>파이썬에서 try-except가 왜 쓰여?</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>단순 설명</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>로지스틱 회귀(Logistic Regression)의 비용 함수를 유도하고, 경사하강법으로 파라미터를 최적화하는 과정을 수식으로 설명하시오.</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>ML 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Design a URL shortening service like bit.ly that handles 100 million URLs with sub-millisecond redirect latency. Include database schema, caching strategy, and hash collision handling.</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>시스템 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>파이썬 GIL(Global Interpreter Lock)의 동작 원리를 설명하고, CPU 바운드 vs I/O 바운드 작업에서 멀티스레딩 성능 차이가 나는 이유를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>파이썬 내부</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Prove the correctness of the merge sort algorithm using mathematical induction, and derive its time complexity recurrence relation using the Master Theorem.</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>알고리즘 증명</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>트랜스포머 모델의 Positional Encoding이 왜 필요한지 수식과 함께 설명하고, 학습 가능한 인코딩과 고정 sin/cos 인코딩의 trade-off를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>NLP 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Analyze how a B-tree maintains balance during insertions and deletions. Prove that the height of a B-tree with n keys and minimum degree t is O(log_t(n)).</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>자료구조 증명</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>쿠버네티스(Kubernetes)에서 Pod 스케줄링 알고리즘을 분석하고, 리소스 제약 조건이 있는 클러스터에서 최적 배치 전략을 설계하시오.</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>클라우드 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Derive the gradient of the cross-entropy loss function with respect to the softmax output layer, and explain why this combination is numerically stable.</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>딥러닝 수학</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>이분 탐색(Binary Search) 알고리즘의 정확성을 루프 불변식(loop invariant)으로 증명하고, 정렬된 배열에서의 시간 복잡도를 엄밀하게 유도하시오.</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>알고리즘 증명</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Compare the architectural differences between BERT, GPT, and T5, analyzing their pre-training objectives, attention patterns, and trade-offs for generation vs. understanding tasks.</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>LLM 아키텍처 비교</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>관계형 데이터베이스의 정규화 과정(1NF~BCNF)을 이상 현상(Anomaly) 관점에서 단계별로 설명하고, 역정규화(Denormalization)가 필요한 상황과 그 trade-off를 논하시오.</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>DB 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Design a rate limiter for a public API that enforces per-user limits (1000 req/min) across a distributed cluster of 50 servers without a centralized bottleneck.</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>분산 시스템 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>확률론에서 중심 극한 정리(CLT)를 엄밀하게 증명하고, 이것이 머신러닝에서 미니배치 학습의 이론적 근거가 되는 방식을 설명하시오.</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>확률 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Analyze the time and space complexity of Dijkstra's algorithm with a binary heap vs. a Fibonacci heap. Explain when the Fibonacci heap version is theoretically superior.</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>알고리즘 분석</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>멀티헤드 어텐션(Multi-Head Attention)이 단일 헤드 어텐션 대비 어떤 표현력을 추가로 갖는지 수식으로 분석하고, 헤드 수와 모델 성능의 관계를 실험적 근거로 설명하시오.</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>1</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>어텐션 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Implement and analyze a concurrent hash map using fine-grained locking. Compare with lock-free approaches using CAS and discuss the ABA problem in detail.</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>동시성 자료구조</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>오토인코더(Autoencoder)의 잠재 공간(latent space) 표현 학습 원리를 설명하고, 이를 이상 탐지(anomaly detection)에 적용할 때의 이론적 근거와 한계를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>1</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>생성 모델</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Analyze the differences between optimistic and pessimistic concurrency control in distributed databases. When does each approach lead to better throughput under high contention?</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>분산 DB 동시성</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>k-means 클러스터링 알고리즘의 수렴성을 증명하고, 초기화 방법(랜덤 vs k-means++)이 최종 결과에 미치는 영향을 이론적·실험적으로 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>비지도 학습 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Design a global payment processing system that handles 10,000 transactions per second with ACID guarantees across multiple currencies and regulatory jurisdictions.</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>대규모 시스템 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>TCP의 혼잡 제어 알고리즘(AIMD, Slow Start, Fast Retransmit)을 분석하고, CUBIC과 BBR이 기존 방식 대비 고대역폭 고지연 네트워크에서 어떻게 성능을 개선하는지 설명하시오.</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>네트워크 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Prove that any comparison-based sorting algorithm requires Ω(n log n) comparisons in the worst case using a decision tree argument.</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>정렬 하한 증명</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>배치 정규화(Batch Normalization)와 레이어 정규화(Layer Normalization)의 수식을 비교하고, 각각이 RNN과 Transformer에 적합한 이유를 gradient flow 관점에서 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>정규화 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Analyze how consistent hashing with virtual nodes solves the hot-spot problem in distributed key-value stores. Derive the expected load imbalance as a function of virtual node count.</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>분산 해싱 분석</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>재귀 하강 파서(Recursive Descent Parser)로 문맥 자유 문법(CFG)을 구현하는 방법을 설명하고, 좌재귀(left recursion) 문제를 해결하기 위한 문법 변환 방법을 논하시오.</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>파서 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Compare dropout, weight decay, and early stopping as regularization techniques. Derive the equivalence between L2 regularization and Gaussian weight priors in a Bayesian framework.</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>정규화 수학</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>링크드 리스트로 LRU 캐시를 O(1) 시간 복잡도로 구현하는 방법을 설계하고, 분산 환경에서 LRU 정책을 유지하는 것이 왜 어려운지 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>캐시 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Analyze the trade-offs between synchronous replication and asynchronous replication in distributed databases. Derive the relationship between replication lag and write throughput.</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>1</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>분산 DB 복제</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>주성분 분석(PCA)의 수학적 원리를 공분산 행렬의 고유값 분해 관점에서 유도하고, SVD와의 관계를 설명하시오. 차원 축소 시 정보 손실량을 정량화하는 방법도 포함하시오.</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>1</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>차원 축소 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Design a distributed tracing system for a microservices architecture with 200 services. Address context propagation, sampling strategies, and storage trade-offs for trace data.</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>관측성 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>소수 판별 알고리즘(Miller-Rabin, AKS)의 동작 원리를 비교하고, RSA 키 생성 과정에서 대형 소수를 효율적으로 생성하는 방법의 확률론적 근거를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>암호학 알고리즘</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Analyze the vanishing and exploding gradient problems in deep RNNs. Derive mathematically why LSTMs mitigate vanishing gradients through their gating mechanism.</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>LSTM 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>그래프에서 최소 신장 트리(MST)를 구하는 Kruskal과 Prim 알고리즘의 정확성을 각각 컷 성질(cut property)과 사이클 성질로 증명하시오.</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>그래프 알고리즘 증명</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Explain the internals of the Linux virtual memory system, including page tables, TLB, huge pages, and how the kernel handles page faults and memory-mapped files.</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>OS 내부</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>모델 압축 기법(Pruning, Quantization, Knowledge Distillation)을 비교하고, 각 방법이 추론 속도와 정확도 trade-off에 미치는 영향을 이론적·실험적으로 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>모델 경량화</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Design a type-safe, zero-overhead optional type for a systems programming language. Analyze how Rust's Option&lt;T&gt; achieves this and compare with nullable pointers in C++.</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>언어 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>해시 테이블에서 충돌 해결 방법(체이닝 vs 개방 주소법)을 평균·최악 시간 복잡도 관점에서 분석하고, 부하율(load factor)이 성능에 미치는 영향을 확률론적으로 유도하시오.</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>해시 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Compare Actor model, CSP, and shared-memory concurrency models. Analyze how Erlang's OTP supervision trees achieve fault tolerance and compare with Go's goroutines.</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>동시성 모델</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>랜덤 포레스트(Random Forest)에서 배깅(Bagging)과 피처 랜덤 샘플링이 분산을 줄이는 이유를 bias-variance decomposition으로 수식 유도하시오.</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>앙상블 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Design a multi-region active-active database architecture that maintains causal consistency while tolerating network partitions. Analyze the implementation using vector clocks.</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>분산 일관성</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>컴파일러의 레지스터 할당 문제를 그래프 색칠 문제(Graph Coloring)로 모델링하는 방법을 설명하고, NP-완전임에도 실용적인 휴리스틱으로 해결하는 방법을 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>컴파일러 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Analyze the security properties of TLS 1.3 compared to TLS 1.2. Explain forward secrecy, the 0-RTT handshake trade-offs, and resistance to downgrade attacks.</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>네트워크 보안</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>몬테카를로 트리 탐색(MCTS) 알고리즘을 UCB1 공식을 중심으로 설명하고, AlphaGo에서 신경망과 결합된 방식이 탐색 효율을 어떻게 향상시키는지 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>강화학습+탐색</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Derive the amortized time complexity of dynamic array resizing using the accounting method and potential method of amortized analysis.</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>분할 상환 분석</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>멀티모달 LLM에서 비전 인코더와 언어 모델을 정렬(alignment)하는 방법을 비교하고(CLIP, BLIP-2, LLaVA), 각 접근법의 데이터 효율성과 성능 trade-off를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>멀티모달 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Analyze how Postgres implements MVCC using transaction IDs, visibility rules, and the clog. Explain how VACUUM reclaims dead tuples and why it's necessary for performance.</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>DB 내부 구조</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>스펙트럼 클러스터링(Spectral Clustering)의 수학적 원리를 그래프 라플라시안 행렬의 고유벡터 분해 관점에서 설명하고, k-means와의 근본적인 차이를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>클러스터링 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Design a zero-downtime database migration strategy for a 10TB production database. Address schema changes, data backfills, dual-write patterns, and rollback procedures.</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>DB 마이그레이션</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>플로이드-워셜(Floyd-Warshall) 알고리즘이 음수 가중치를 처리하는 원리를 동적 프로그래밍 점화식으로 유도하고, 음수 사이클 탐지 방법과 시간 복잡도를 분석하시오.</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>그래프 DP</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Analyze the theoretical and practical differences between synchronous SGD and asynchronous SGD in distributed training. Derive the convergence guarantees and explain gradient staleness effects.</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>1</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>분산 학습 이론</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>